<commit_message>
refactored apiKeys table structure and added new route files for loans and user management
</commit_message>
<xml_diff>
--- a/backendV2/scheme.xlsx
+++ b/backendV2/scheme.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/theis/Documents/Dock folder/Repos/borrow-system/backend/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/theis/Documents/Dock folder/Repos/borrow-system/backendV2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA1E0B56-988D-B248-AE3D-F780B184C861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F286EB7-48F1-3747-A083-D6C28D728DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4340" yWindow="-28180" windowWidth="51200" windowHeight="24540" activeTab="1" xr2:uid="{C8FDF089-DA29-D94D-9C59-AF6D7D2004E6}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="20860" activeTab="3" xr2:uid="{C8FDF089-DA29-D94D-9C59-AF6D7D2004E6}"/>
   </bookViews>
   <sheets>
     <sheet name="users" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>id</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>note</t>
+  </si>
+  <si>
+    <t>last_used_at</t>
   </si>
 </sst>
 </file>
@@ -547,6 +550,8 @@
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -640,16 +645,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EC061F4-246A-8B47-B471-2C9717CEC715}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -660,6 +666,9 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
began to refactor backend
</commit_message>
<xml_diff>
--- a/backendV2/scheme.xlsx
+++ b/backendV2/scheme.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/theis/Documents/Dock folder/Repos/borrow-system/backendV2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F286EB7-48F1-3747-A083-D6C28D728DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4AFDC6A-4C65-B44F-B038-F25AE75444FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="20860" activeTab="3" xr2:uid="{C8FDF089-DA29-D94D-9C59-AF6D7D2004E6}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="20860" xr2:uid="{C8FDF089-DA29-D94D-9C59-AF6D7D2004E6}"/>
   </bookViews>
   <sheets>
     <sheet name="users" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>last_used_at</t>
+  </si>
+  <si>
+    <t>email</t>
   </si>
 </sst>
 </file>
@@ -488,21 +491,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C45E80-8993-894A-A364-6FA07B6EC85C}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,21 +517,24 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>